<commit_message>
Finalize SwiftLog Week 5 ML engineering project
</commit_message>
<xml_diff>
--- a/Models/Model_Comparison.xlsx
+++ b/Models/Model_Comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="34">
   <si>
     <t>Problem</t>
   </si>
@@ -49,6 +49,21 @@
     <t>ROC_AUC</t>
   </si>
   <si>
+    <t>Test_Accuracy</t>
+  </si>
+  <si>
+    <t>Test_Precision</t>
+  </si>
+  <si>
+    <t>Test_Recall</t>
+  </si>
+  <si>
+    <t>Test_F1</t>
+  </si>
+  <si>
+    <t>Test_ROC_AUC</t>
+  </si>
+  <si>
     <t>MAE</t>
   </si>
   <si>
@@ -56,6 +71,15 @@
   </si>
   <si>
     <t>R2</t>
+  </si>
+  <si>
+    <t>Test_MAE</t>
+  </si>
+  <si>
+    <t>Test_RMSE</t>
+  </si>
+  <si>
+    <t>Test_R2</t>
   </si>
   <si>
     <t>Delivery Delay Classification</t>
@@ -98,16 +122,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -123,7 +139,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -131,30 +147,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -449,59 +447,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:22">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C2">
         <v>5000</v>
@@ -516,27 +538,42 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>0.829</v>
+        <v>0.827</v>
       </c>
       <c r="H2">
-        <v>0.8829902491874323</v>
+        <v>0.8802588996763754</v>
       </c>
       <c r="I2">
-        <v>0.928246013667426</v>
+        <v>0.929384965831435</v>
       </c>
       <c r="J2">
-        <v>0.9050527484730705</v>
+        <v>0.9041551246537396</v>
       </c>
       <c r="K2">
-        <v>0.5118936480077673</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>0.496289069793495</v>
+      </c>
+      <c r="L2">
+        <v>0.827</v>
+      </c>
+      <c r="M2">
+        <v>0.8770053475935828</v>
+      </c>
+      <c r="N2">
+        <v>0.9339407744874715</v>
+      </c>
+      <c r="O2">
+        <v>0.9045780474351903</v>
+      </c>
+      <c r="P2">
+        <v>0.5164681280107547</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C3">
         <v>5000</v>
@@ -551,27 +588,27 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>0.542</v>
+        <v>0.597</v>
       </c>
       <c r="H3">
-        <v>0.8763440860215054</v>
+        <v>0.8861788617886179</v>
       </c>
       <c r="I3">
-        <v>0.5569476082004556</v>
+        <v>0.6207289293849658</v>
       </c>
       <c r="J3">
-        <v>0.6810584958217271</v>
+        <v>0.7300736771600804</v>
       </c>
       <c r="K3">
-        <v>0.4866453190933194</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
+        <v>0.5459175099891707</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -586,27 +623,27 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>0.523</v>
+        <v>0.527</v>
       </c>
       <c r="H4">
-        <v>0.8719851576994434</v>
+        <v>0.87569573283859</v>
       </c>
       <c r="I4">
-        <v>0.5353075170842825</v>
+        <v>0.5375854214123007</v>
       </c>
       <c r="J4">
-        <v>0.6633733239237827</v>
+        <v>0.666196189131969</v>
       </c>
       <c r="K4">
-        <v>0.4754471787594757</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+        <v>0.4840406661936592</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C5">
         <v>5000</v>
@@ -621,27 +658,42 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>0.538</v>
+        <v>0.47</v>
       </c>
       <c r="H5">
-        <v>0.09846827133479212</v>
+        <v>0.09479553903345725</v>
       </c>
       <c r="I5">
-        <v>0.4736842105263158</v>
+        <v>0.5425531914893617</v>
       </c>
       <c r="J5">
-        <v>0.1630434782608696</v>
+        <v>0.1613924050632911</v>
       </c>
       <c r="K5">
-        <v>0.4875952311718523</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
+        <v>0.4810776854069795</v>
+      </c>
+      <c r="L5">
+        <v>0.421</v>
+      </c>
+      <c r="M5">
+        <v>0.08561643835616438</v>
+      </c>
+      <c r="N5">
+        <v>0.5263157894736842</v>
+      </c>
+      <c r="O5">
+        <v>0.1472754050073638</v>
+      </c>
+      <c r="P5">
+        <v>0.4757313172433847</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C6">
         <v>5000</v>
@@ -656,27 +708,27 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>0.421</v>
+        <v>0.554</v>
       </c>
       <c r="H6">
-        <v>0.08561643835616438</v>
+        <v>0.09069767441860466</v>
       </c>
       <c r="I6">
-        <v>0.5263157894736842</v>
+        <v>0.4148936170212766</v>
       </c>
       <c r="J6">
-        <v>0.1472754050073638</v>
+        <v>0.1488549618320611</v>
       </c>
       <c r="K6">
-        <v>0.4757313172433847</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
+        <v>0.4943168474942464</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C7">
         <v>5000</v>
@@ -691,27 +743,27 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>0.88</v>
+        <v>0.876</v>
       </c>
       <c r="H7">
-        <v>0.09677419354838709</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>0.03157894736842105</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>0.04761904761904762</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>0.5089619075312591</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
+        <v>0.5263961298201117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C8">
         <v>8250</v>
@@ -725,22 +777,31 @@
       <c r="F8" t="b">
         <v>1</v>
       </c>
-      <c r="L8">
+      <c r="Q8">
+        <v>6.403765296170344</v>
+      </c>
+      <c r="R8">
+        <v>7.956981450540439</v>
+      </c>
+      <c r="S8">
+        <v>-0.02826315793925072</v>
+      </c>
+      <c r="T8">
         <v>6.52383479099333</v>
       </c>
-      <c r="M8">
+      <c r="U8">
         <v>8.077777650609818</v>
       </c>
-      <c r="N8">
+      <c r="V8">
         <v>-0.01397950676738624</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:22">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C9">
         <v>8250</v>
@@ -754,22 +815,22 @@
       <c r="F9" t="b">
         <v>0</v>
       </c>
-      <c r="L9">
-        <v>6.657535776672379</v>
-      </c>
-      <c r="M9">
-        <v>8.485197174750331</v>
-      </c>
-      <c r="N9">
-        <v>-0.1188433009910457</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
+      <c r="Q9">
+        <v>6.597686973659411</v>
+      </c>
+      <c r="R9">
+        <v>8.401859113827348</v>
+      </c>
+      <c r="S9">
+        <v>-0.1464585933889377</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C10">
         <v>8250</v>
@@ -783,22 +844,22 @@
       <c r="F10" t="b">
         <v>0</v>
       </c>
-      <c r="L10">
-        <v>6.612884548781703</v>
-      </c>
-      <c r="M10">
-        <v>8.205114995326459</v>
-      </c>
-      <c r="N10">
-        <v>-0.0462000410504475</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
+      <c r="Q10">
+        <v>6.716671381465901</v>
+      </c>
+      <c r="R10">
+        <v>8.337240191028179</v>
+      </c>
+      <c r="S10">
+        <v>-0.1288915212723023</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C11">
         <v>6000</v>
@@ -812,22 +873,31 @@
       <c r="F11" t="b">
         <v>0</v>
       </c>
-      <c r="L11">
+      <c r="Q11">
+        <v>3160.402387603192</v>
+      </c>
+      <c r="R11">
+        <v>4082.077920856409</v>
+      </c>
+      <c r="S11">
+        <v>0.001432104011237167</v>
+      </c>
+      <c r="T11">
         <v>2990.706372983079</v>
       </c>
-      <c r="M11">
+      <c r="U11">
         <v>3757.004105184792</v>
       </c>
-      <c r="N11">
+      <c r="V11">
         <v>-0.06860620869491374</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:22">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C12">
         <v>6000</v>
@@ -841,22 +911,22 @@
       <c r="F12" t="b">
         <v>0</v>
       </c>
-      <c r="L12">
-        <v>3133.165306934514</v>
-      </c>
-      <c r="M12">
-        <v>4164.917948928041</v>
-      </c>
-      <c r="N12">
-        <v>-0.3132495296375171</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
+      <c r="Q12">
+        <v>3290.482736255518</v>
+      </c>
+      <c r="R12">
+        <v>4446.408837890341</v>
+      </c>
+      <c r="S12">
+        <v>-0.1847693314833916</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C13">
         <v>6000</v>
@@ -870,14 +940,14 @@
       <c r="F13" t="b">
         <v>0</v>
       </c>
-      <c r="L13">
-        <v>3034.185432860818</v>
-      </c>
-      <c r="M13">
-        <v>3837.693256126995</v>
-      </c>
-      <c r="N13">
-        <v>-0.1150000114782266</v>
+      <c r="Q13">
+        <v>3161.887587356699</v>
+      </c>
+      <c r="R13">
+        <v>4136.253897014216</v>
+      </c>
+      <c r="S13">
+        <v>-0.02524910074539544</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix report generation and refresh Week 5 deliverables
</commit_message>
<xml_diff>
--- a/Models/Model_Comparison.xlsx
+++ b/Models/Model_Comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="41">
   <si>
     <t>Problem</t>
   </si>
@@ -28,25 +28,40 @@
     <t>Features</t>
   </si>
   <si>
+    <t>Train_Rows</t>
+  </si>
+  <si>
+    <t>Validation_Rows</t>
+  </si>
+  <si>
+    <t>Test_Rows</t>
+  </si>
+  <si>
     <t>Selected</t>
   </si>
   <si>
     <t>Tuned</t>
   </si>
   <si>
-    <t>Accuracy</t>
-  </si>
-  <si>
-    <t>Precision</t>
-  </si>
-  <si>
-    <t>Recall</t>
-  </si>
-  <si>
-    <t>F1</t>
-  </si>
-  <si>
-    <t>ROC_AUC</t>
+    <t>Selection_Basis</t>
+  </si>
+  <si>
+    <t>Validation_Accuracy</t>
+  </si>
+  <si>
+    <t>Validation_Precision</t>
+  </si>
+  <si>
+    <t>Validation_Recall</t>
+  </si>
+  <si>
+    <t>Validation_F1</t>
+  </si>
+  <si>
+    <t>Validation_ROC_AUC</t>
+  </si>
+  <si>
+    <t>Tuned_Validation_Score</t>
   </si>
   <si>
     <t>Test_Accuracy</t>
@@ -64,13 +79,13 @@
     <t>Test_ROC_AUC</t>
   </si>
   <si>
-    <t>MAE</t>
-  </si>
-  <si>
-    <t>RMSE</t>
-  </si>
-  <si>
-    <t>R2</t>
+    <t>Validation_MAE</t>
+  </si>
+  <si>
+    <t>Validation_RMSE</t>
+  </si>
+  <si>
+    <t>Validation_R2</t>
   </si>
   <si>
     <t>Test_MAE</t>
@@ -116,6 +131,12 @@
   </si>
   <si>
     <t>Random Forest Regressor</t>
+  </si>
+  <si>
+    <t>Validation F1</t>
+  </si>
+  <si>
+    <t>Validation RMSE</t>
   </si>
 </sst>
 </file>
@@ -447,10 +468,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:22">
+    <row r="1" spans="1:27">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -517,13 +538,28 @@
       <c r="V1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:22">
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C2">
         <v>5000</v>
@@ -531,49 +567,64 @@
       <c r="D2">
         <v>7</v>
       </c>
-      <c r="E2" t="b">
+      <c r="E2">
+        <v>3000</v>
+      </c>
+      <c r="F2">
+        <v>1000</v>
+      </c>
+      <c r="G2">
+        <v>1000</v>
+      </c>
+      <c r="H2" t="b">
         <v>1</v>
       </c>
-      <c r="F2" t="b">
+      <c r="I2" t="b">
         <v>1</v>
       </c>
-      <c r="G2">
-        <v>0.827</v>
-      </c>
-      <c r="H2">
-        <v>0.8802588996763754</v>
-      </c>
-      <c r="I2">
-        <v>0.929384965831435</v>
-      </c>
-      <c r="J2">
-        <v>0.9041551246537396</v>
+      <c r="J2" t="s">
+        <v>39</v>
       </c>
       <c r="K2">
-        <v>0.496289069793495</v>
+        <v>0.831</v>
       </c>
       <c r="L2">
-        <v>0.827</v>
+        <v>0.8807733619763695</v>
       </c>
       <c r="M2">
-        <v>0.8770053475935828</v>
+        <v>0.9339407744874715</v>
       </c>
       <c r="N2">
-        <v>0.9339407744874715</v>
+        <v>0.9065782200110558</v>
       </c>
       <c r="O2">
-        <v>0.9045780474351903</v>
+        <v>0.4995192128160125</v>
       </c>
       <c r="P2">
-        <v>0.5164681280107547</v>
-      </c>
-    </row>
-    <row r="3" spans="1:22">
+        <v>0.9207383279044516</v>
+      </c>
+      <c r="Q2">
+        <v>0.852</v>
+      </c>
+      <c r="R2">
+        <v>0.8794178794178794</v>
+      </c>
+      <c r="S2">
+        <v>0.9635535307517085</v>
+      </c>
+      <c r="T2">
+        <v>0.9195652173913044</v>
+      </c>
+      <c r="U2">
+        <v>0.5058301280854401</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C3">
         <v>5000</v>
@@ -581,34 +632,46 @@
       <c r="D3">
         <v>7</v>
       </c>
-      <c r="E3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F3" t="b">
-        <v>0</v>
+      <c r="E3">
+        <v>3000</v>
+      </c>
+      <c r="F3">
+        <v>1000</v>
       </c>
       <c r="G3">
+        <v>1000</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3">
         <v>0.597</v>
       </c>
-      <c r="H3">
+      <c r="L3">
         <v>0.8861788617886179</v>
       </c>
-      <c r="I3">
+      <c r="M3">
         <v>0.6207289293849658</v>
       </c>
-      <c r="J3">
+      <c r="N3">
         <v>0.7300736771600804</v>
       </c>
-      <c r="K3">
+      <c r="O3">
         <v>0.5459175099891707</v>
       </c>
     </row>
-    <row r="4" spans="1:22">
+    <row r="4" spans="1:27">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -616,34 +679,46 @@
       <c r="D4">
         <v>7</v>
       </c>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" t="b">
-        <v>0</v>
+      <c r="E4">
+        <v>3000</v>
+      </c>
+      <c r="F4">
+        <v>1000</v>
       </c>
       <c r="G4">
+        <v>1000</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K4">
         <v>0.527</v>
       </c>
-      <c r="H4">
+      <c r="L4">
         <v>0.87569573283859</v>
       </c>
-      <c r="I4">
+      <c r="M4">
         <v>0.5375854214123007</v>
       </c>
-      <c r="J4">
+      <c r="N4">
         <v>0.666196189131969</v>
       </c>
-      <c r="K4">
+      <c r="O4">
         <v>0.4840406661936592</v>
       </c>
     </row>
-    <row r="5" spans="1:22">
+    <row r="5" spans="1:27">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C5">
         <v>5000</v>
@@ -651,49 +726,61 @@
       <c r="D5">
         <v>10</v>
       </c>
-      <c r="E5" t="b">
+      <c r="E5">
+        <v>3000</v>
+      </c>
+      <c r="F5">
+        <v>1000</v>
+      </c>
+      <c r="G5">
+        <v>1000</v>
+      </c>
+      <c r="H5" t="b">
         <v>1</v>
       </c>
-      <c r="F5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0.47</v>
-      </c>
-      <c r="H5">
-        <v>0.09479553903345725</v>
-      </c>
-      <c r="I5">
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5">
+        <v>0.472</v>
+      </c>
+      <c r="L5">
+        <v>0.09514925373134328</v>
+      </c>
+      <c r="M5">
         <v>0.5425531914893617</v>
       </c>
-      <c r="J5">
-        <v>0.1613924050632911</v>
-      </c>
-      <c r="K5">
-        <v>0.4810776854069795</v>
-      </c>
-      <c r="L5">
-        <v>0.421</v>
-      </c>
-      <c r="M5">
-        <v>0.08561643835616438</v>
-      </c>
       <c r="N5">
+        <v>0.1619047619047619</v>
+      </c>
+      <c r="O5">
+        <v>0.4829681555586869</v>
+      </c>
+      <c r="Q5">
+        <v>0.424</v>
+      </c>
+      <c r="R5">
+        <v>0.08605851979345955</v>
+      </c>
+      <c r="S5">
         <v>0.5263157894736842</v>
       </c>
-      <c r="O5">
-        <v>0.1472754050073638</v>
-      </c>
-      <c r="P5">
-        <v>0.4757313172433847</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22">
+      <c r="T5">
+        <v>0.1479289940828402</v>
+      </c>
+      <c r="U5">
+        <v>0.478261122419308</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C6">
         <v>5000</v>
@@ -701,34 +788,46 @@
       <c r="D6">
         <v>10</v>
       </c>
-      <c r="E6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F6" t="b">
-        <v>0</v>
+      <c r="E6">
+        <v>3000</v>
+      </c>
+      <c r="F6">
+        <v>1000</v>
       </c>
       <c r="G6">
+        <v>1000</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="s">
+        <v>39</v>
+      </c>
+      <c r="K6">
         <v>0.554</v>
       </c>
-      <c r="H6">
+      <c r="L6">
         <v>0.09069767441860466</v>
       </c>
-      <c r="I6">
+      <c r="M6">
         <v>0.4148936170212766</v>
       </c>
-      <c r="J6">
+      <c r="N6">
         <v>0.1488549618320611</v>
       </c>
-      <c r="K6">
+      <c r="O6">
         <v>0.4943168474942464</v>
       </c>
     </row>
-    <row r="7" spans="1:22">
+    <row r="7" spans="1:27">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C7">
         <v>5000</v>
@@ -736,34 +835,46 @@
       <c r="D7">
         <v>10</v>
       </c>
-      <c r="E7" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" t="b">
-        <v>0</v>
+      <c r="E7">
+        <v>3000</v>
+      </c>
+      <c r="F7">
+        <v>1000</v>
       </c>
       <c r="G7">
-        <v>0.876</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
+        <v>1000</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="s">
+        <v>39</v>
       </c>
       <c r="K7">
-        <v>0.5263961298201117</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22">
+        <v>0.881</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0.5297543563007844</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C8">
         <v>8250</v>
@@ -771,37 +882,52 @@
       <c r="D8">
         <v>9</v>
       </c>
-      <c r="E8" t="b">
+      <c r="E8">
+        <v>4750</v>
+      </c>
+      <c r="F8">
+        <v>1750</v>
+      </c>
+      <c r="G8">
+        <v>1750</v>
+      </c>
+      <c r="H8" t="b">
         <v>1</v>
       </c>
-      <c r="F8" t="b">
+      <c r="I8" t="b">
         <v>1</v>
       </c>
-      <c r="Q8">
-        <v>6.403765296170344</v>
-      </c>
-      <c r="R8">
-        <v>7.956981450540439</v>
-      </c>
-      <c r="S8">
-        <v>-0.02826315793925072</v>
-      </c>
-      <c r="T8">
-        <v>6.52383479099333</v>
-      </c>
-      <c r="U8">
-        <v>8.077777650609818</v>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+      <c r="P8">
+        <v>-7.911034278253315</v>
       </c>
       <c r="V8">
-        <v>-0.01397950676738624</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22">
+        <v>6.39942397542238</v>
+      </c>
+      <c r="W8">
+        <v>7.95133509130753</v>
+      </c>
+      <c r="X8">
+        <v>-0.02680434262541698</v>
+      </c>
+      <c r="Y8">
+        <v>6.527953990751539</v>
+      </c>
+      <c r="Z8">
+        <v>8.069800718234047</v>
+      </c>
+      <c r="AA8">
+        <v>-0.01197785419118746</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C9">
         <v>8250</v>
@@ -809,28 +935,40 @@
       <c r="D9">
         <v>9</v>
       </c>
-      <c r="E9" t="b">
-        <v>0</v>
-      </c>
-      <c r="F9" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q9">
+      <c r="E9">
+        <v>4750</v>
+      </c>
+      <c r="F9">
+        <v>1750</v>
+      </c>
+      <c r="G9">
+        <v>1750</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" t="s">
+        <v>40</v>
+      </c>
+      <c r="V9">
         <v>6.597686973659411</v>
       </c>
-      <c r="R9">
+      <c r="W9">
         <v>8.401859113827348</v>
       </c>
-      <c r="S9">
+      <c r="X9">
         <v>-0.1464585933889377</v>
       </c>
     </row>
-    <row r="10" spans="1:22">
+    <row r="10" spans="1:27">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C10">
         <v>8250</v>
@@ -838,28 +976,40 @@
       <c r="D10">
         <v>9</v>
       </c>
-      <c r="E10" t="b">
-        <v>0</v>
-      </c>
-      <c r="F10" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q10">
+      <c r="E10">
+        <v>4750</v>
+      </c>
+      <c r="F10">
+        <v>1750</v>
+      </c>
+      <c r="G10">
+        <v>1750</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" t="s">
+        <v>40</v>
+      </c>
+      <c r="V10">
         <v>6.716671381465901</v>
       </c>
-      <c r="R10">
+      <c r="W10">
         <v>8.337240191028179</v>
       </c>
-      <c r="S10">
+      <c r="X10">
         <v>-0.1288915212723023</v>
       </c>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:27">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C11">
         <v>6000</v>
@@ -867,37 +1017,49 @@
       <c r="D11">
         <v>6</v>
       </c>
-      <c r="E11" t="b">
+      <c r="E11">
+        <v>3000</v>
+      </c>
+      <c r="F11">
+        <v>1000</v>
+      </c>
+      <c r="G11">
+        <v>2000</v>
+      </c>
+      <c r="H11" t="b">
         <v>1</v>
       </c>
-      <c r="F11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q11">
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" t="s">
+        <v>40</v>
+      </c>
+      <c r="V11">
         <v>3160.402387603192</v>
       </c>
-      <c r="R11">
+      <c r="W11">
         <v>4082.077920856409</v>
       </c>
-      <c r="S11">
+      <c r="X11">
         <v>0.001432104011237167</v>
       </c>
-      <c r="T11">
+      <c r="Y11">
         <v>2990.706372983079</v>
       </c>
-      <c r="U11">
+      <c r="Z11">
         <v>3757.004105184792</v>
       </c>
-      <c r="V11">
+      <c r="AA11">
         <v>-0.06860620869491374</v>
       </c>
     </row>
-    <row r="12" spans="1:22">
+    <row r="12" spans="1:27">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C12">
         <v>6000</v>
@@ -905,28 +1067,40 @@
       <c r="D12">
         <v>6</v>
       </c>
-      <c r="E12" t="b">
-        <v>0</v>
-      </c>
-      <c r="F12" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q12">
+      <c r="E12">
+        <v>3000</v>
+      </c>
+      <c r="F12">
+        <v>1000</v>
+      </c>
+      <c r="G12">
+        <v>2000</v>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" t="s">
+        <v>40</v>
+      </c>
+      <c r="V12">
         <v>3290.482736255518</v>
       </c>
-      <c r="R12">
+      <c r="W12">
         <v>4446.408837890341</v>
       </c>
-      <c r="S12">
+      <c r="X12">
         <v>-0.1847693314833916</v>
       </c>
     </row>
-    <row r="13" spans="1:22">
+    <row r="13" spans="1:27">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C13">
         <v>6000</v>
@@ -934,20 +1108,32 @@
       <c r="D13">
         <v>6</v>
       </c>
-      <c r="E13" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q13">
-        <v>3161.887587356699</v>
-      </c>
-      <c r="R13">
-        <v>4136.253897014216</v>
-      </c>
-      <c r="S13">
-        <v>-0.02524910074539544</v>
+      <c r="E13">
+        <v>3000</v>
+      </c>
+      <c r="F13">
+        <v>1000</v>
+      </c>
+      <c r="G13">
+        <v>2000</v>
+      </c>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J13" t="s">
+        <v>40</v>
+      </c>
+      <c r="V13">
+        <v>3154.34771064244</v>
+      </c>
+      <c r="W13">
+        <v>4127.370499590647</v>
+      </c>
+      <c r="X13">
+        <v>-0.02084999218644334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>